<commit_message>
Review sheet: remove leftover yellow marks in Portfolio Journey savings rows
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K66kUEEu3eBV9D8wyumc1E
</commit_message>
<xml_diff>
--- a/public/templates/client-review.xlsx
+++ b/public/templates/client-review.xlsx
@@ -32353,7 +32353,7 @@
       <c r="F96" s="191"/>
       <c r="G96" s="191"/>
       <c r="H96" s="191"/>
-      <c r="I96" s="356"/>
+      <c r="I96" s="191"/>
       <c r="J96" s="191"/>
       <c r="K96" s="191"/>
       <c r="L96" s="191"/>
@@ -32810,7 +32810,7 @@
       <c r="F102" s="191"/>
       <c r="G102" s="191"/>
       <c r="H102" s="191"/>
-      <c r="I102" s="356"/>
+      <c r="I102" s="191"/>
       <c r="J102" s="191"/>
       <c r="K102" s="191"/>
       <c r="L102" s="191"/>
@@ -33428,7 +33428,7 @@
       <c r="F110" s="191"/>
       <c r="G110" s="191"/>
       <c r="H110" s="191"/>
-      <c r="I110" s="356"/>
+      <c r="I110" s="191"/>
       <c r="J110" s="191"/>
       <c r="K110" s="191"/>
       <c r="L110" s="191"/>
@@ -33605,7 +33605,7 @@
       <c r="F112" s="191"/>
       <c r="G112" s="191"/>
       <c r="H112" s="191"/>
-      <c r="I112" s="356"/>
+      <c r="I112" s="191"/>
       <c r="J112" s="191"/>
       <c r="K112" s="191"/>
       <c r="L112" s="191"/>
@@ -33695,7 +33695,7 @@
       <c r="F114" s="191"/>
       <c r="G114" s="191"/>
       <c r="H114" s="191"/>
-      <c r="I114" s="356"/>
+      <c r="I114" s="191"/>
       <c r="J114" s="191"/>
       <c r="K114" s="191"/>
       <c r="L114" s="191"/>
@@ -33983,7 +33983,7 @@
       <c r="F118" s="191"/>
       <c r="G118" s="191"/>
       <c r="H118" s="191"/>
-      <c r="I118" s="356"/>
+      <c r="I118" s="191"/>
       <c r="J118" s="191"/>
       <c r="K118" s="191"/>
       <c r="L118" s="191"/>
@@ -34044,7 +34044,7 @@
       <c r="F119" s="191"/>
       <c r="G119" s="191"/>
       <c r="H119" s="191"/>
-      <c r="I119" s="356"/>
+      <c r="I119" s="191"/>
       <c r="J119" s="191"/>
       <c r="K119" s="191"/>
       <c r="L119" s="191"/>

</xml_diff>